<commit_message>
Add manual commands / server & database change runbook to work log
New "Manual Commands & Server" sheet in the QA/dev Excel work log,
aimed at teammates setting up a new environment or deploying this
branch: a MUST-RUN section for the ewaybilldate database column that
git can't track, a from-zero environment setup checklist (PHP/MySQL/
Composer install, DB creation, SQL import, .env config, and a note
that the document root must point at the repo root rather than a
public/ subfolder), and a clearly separated list of local-dev-only
conveniences (build/ symlink, router.php, SonarQube container) that
do NOT need to be replicated on a real server.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-Dev-Work-Log.xlsx
+++ b/docs/QA-Dev-Work-Log.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sonar Findings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Bugs Fixed" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Smoke Test Results" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Known Issues (Not Fixed)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Manual Commands &amp; Server" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sonar Findings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Bugs Fixed" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Smoke Test Results" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Known Issues (Not Fixed)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +60,20 @@
       <sz val="10"/>
     </font>
     <font>
+      <name val="Courier New"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C6500"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0052514E"/>
+      <sz val="12"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
   </fonts>
@@ -76,7 +91,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9F2D9"/>
+        <fgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
     <fill>
@@ -91,7 +106,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
+        <fgColor rgb="00D9F2D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -121,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -134,28 +149,43 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -521,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -584,7 +614,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Manual Commands &amp; Server</t>
         </is>
       </c>
     </row>
@@ -701,162 +731,208 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>7. QA: smoke testing</t>
+          <t>6b. Database schema change</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Hit all 34 application routes with an authenticated session</t>
+          <t>Added invoice.ewaybilldate column directly via ALTER TABLE — required for invoice creation to work at all</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>27 pass, 7 fail (all pre-existing, documented, none caused by this work)</t>
+          <t>Applied to local dev DB only — MUST be applied manually to any other environment</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Smoke Test Results</t>
+          <t>Manual Commands &amp; Server</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>8. QA: functional testing</t>
+          <t>7. QA: smoke testing</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>End-to-end tested invoice creation, payment recording, inventory update, product creation against real form submissions</t>
+          <t>Hit all 34 application routes with an authenticated session</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>All 5 core flows verified passing after fixes</t>
+          <t>27 pass, 7 fail (all pre-existing, documented, none caused by this work)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Bugs Fixed</t>
+          <t>Smoke Test Results</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>9. Known issues (not fixed)</t>
+          <t>8. QA: functional testing</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Documented real, confirmed bugs found along the way that were out of scope for this pass</t>
+          <t>End-to-end tested invoice creation, payment recording, inventory update, product creation against real form submissions</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>5 issues logged for a future scoping decision</t>
+          <t>All 5 core flows verified passing after fixes</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Known Issues (Not Fixed)</t>
+          <t>Bugs Fixed</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>9. Known issues (not fixed)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Documented real, confirmed bugs found along the way that were out of scope for this pass</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>5 issues logged for a future scoping decision</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Known Issues (Not Fixed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>10. Git</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Committed and pushed all fixes across two commits to origin/meet-update</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Committed and pushed all fixes across three commits to origin/meet-update</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Pushed — see commit log below</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Commit log (this repo, branch meet-update)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Commit</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Message</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>4c39c24</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Initial project import for meet-update</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>41d6dab</t>
+          <t>4c39c24</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Fix Sonar Blocker and Critical issues (backend + frontend)</t>
+          <t>Initial project import for meet-update</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>41d6dab</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Fix Sonar Blocker and Critical issues (backend + frontend)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
           <t>b4e5550</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Fix Sonar High/Medium issues and critical invoice/payment bugs</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>⚠ Manual step required outside git</t>
-        </is>
-      </c>
-    </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>e729fa1</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Add QA/dev work log spreadsheet documenting the full fix pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>(this commit)</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Add manual commands / server &amp; database change runbook to the work log</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>⚠ Manual step required outside git — see 'Manual Commands &amp; Server' sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>A database column (invoice.ewaybilldate) was added directly via ALTER TABLE on the local dev DB, because this database predates Laravel's migration system (imported from a raw SQL dump, no migrations table). This is NOT captured by any git commit — it must be applied by hand to any other environment (staging/production/teammate's machine):</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>ALTER TABLE invoice ADD COLUMN ewaybilldate DATE NULL AFTER ewaybillno;</t>
         </is>
@@ -872,6 +948,500 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Manual Commands &amp; Server / Database Changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Everything outside git — run these when setting up a new environment or deploying. NOT auto-applied by pulling the branch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>🔴 MUST RUN on every environment (staging / production / a teammate's machine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Command / Change</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Where</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>ALTER TABLE invoice ADD COLUMN ewaybilldate DATE NULL AFTER ewaybillno;</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>MySQL, on the application database</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Column the app code has always expected but was never created. Without it, invoice creation fails (HTTP 500) on every submission — see Bugs Fixed sheet, bug #1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>🟡 Fresh environment / new server setup (from zero)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Command</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Where</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>1. Install PHP 8.2</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>brew install php@8.2   (or apt/yum equivalent on Linux servers)</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Server / host machine</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>composer.json requires "php": "^8.1"; app was built and tested against 8.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>2. Install MySQL</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>brew install mysql   (most hosts already provide this)</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Server / host machine</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Application database engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>3. Install Composer</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>brew install composer</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Server / host machine</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>PHP dependency manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>4. Install PHP dependencies</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>composer install</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Project root</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Installs vendor/ — Laravel framework + packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>5. Install JS dependencies</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>npm install</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Project root</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Only needed if rebuilding frontend assets; the compiled build/ folder is already committed to the repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>6. Create the database + user</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>CREATE DATABASE u411614341_Invoice; CREATE USER 'u411614341_invoice'@'...' IDENTIFIED BY '...'; GRANT ALL PRIVILEGES ON u411614341_Invoice.* TO ...;</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>MySQL</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Matches the credentials already configured in .env — see .env.example for the expected variable names</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>7. Import the database schema + data</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>mysql -u root u411614341_Invoice &lt; "u411614341_Invoice (2).sql"</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>MySQL, from the project root</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Base schema and any seed data. This SQL dump does not include the invoice/customer/product tables' full production data — see Notes below</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>8. Apply the ewaybilldate fix</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>See the MUST RUN row above</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>MySQL</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Required — the SQL dump does not include this column</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>9. Configure environment</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Copy .env.example to .env, set DB_* credentials, APP_URL, APP_KEY</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Project root</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>php artisan key:generate if APP_KEY is blank</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>10. Set the web server document root</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Point the web server's document root at the PROJECT ROOT itself, not a public/ subfolder</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Web server config (Apache/Nginx/hosting panel)</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>This app is a shared-hosting style deployment — index.php, vendor/, bootstrap/ all sit at the repo root (see Notes below). This is NOT the standard Laravel public/ layout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>⚪ Local development convenience only — do NOT need these on a real server</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Command / File</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Why it's dev-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>public/build symlink</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>ln -s ../build public/build</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Lets the built-in PHP dev server find compiled CSS/JS at the URL path Blade templates expect</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>Only needed for `php artisan serve` / `php -S` style local testing. A real Apache/Nginx host serving the whole repo as document root already resolves build/ at the correct path without this symlink.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>router.php</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Custom router script for PHP's built-in server, not part of the Laravel app</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>Makes `php -S 127.0.0.1:8000 router.php` correctly serve static files from the repo root instead of expecting a public/ folder</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>Apache/Nginx don't need a router script — they're configured via vhost/.htaccess instead. Untracked in git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>sonar-project.properties</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>SonarQube scanner config</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>Lets a teammate re-run the same static-analysis scan locally</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>Not part of the running application; safe to keep or delete</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>Local SonarQube (Docker)</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>docker run -d --name sonarqube -p 9000:9000 sonarqube:community</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>Ran a local code-quality dashboard for the Sonar cleanup pass</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>One-off analysis tooling, not part of the deployed app. See the Sonar Findings sheet for results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>• Document root: this repo is deployed shared-hosting style — index.php, vendor/, bootstrap/, .env all sit directly at the project root (not inside a public/ folder as a standard Laravel app would). Confirm the hosting panel / vhost config points at the repo root, not a public/ subfolder that doesn't functionally exist here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>• The imported SQL dump (u411614341_Invoice (2).sql) is a partial export — some tables (invoice, customer) had little or no data at the time of import, which is why several bugs in the Bugs Fixed sheet only surfaced during live functional testing rather than on page load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>• No other schema changes were made this pass beyond the ewaybilldate column. All other fixes were application code only (see Bugs Fixed and Sonar Findings sheets).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>• No new database tables were created and no existing tables were dropped or renamed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A32:D32"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -935,130 +1505,130 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Blocker (Must-Fix)</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Dead IE8/9 CSS hack in vendor flatpickr theme file — removed, zero visual change</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="18" t="n">
         <v>59</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="18" t="n">
         <v>57</v>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>2 remaining are stock Laravel config scaffolding (127.0.0.1 / log path duplication) — won't-fix by design, matches every fresh Laravel install</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>High (Major)</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="12" t="n">
         <v>497</v>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="12" t="n">
         <v>431</v>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="12" t="n">
         <v>66</v>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>Partially fixed</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Remaining 431 dominated by false positives: 361 icon-font CSS declarations, 44 vendor-plugin duplicate CSS selectors (too risky to merge without visual regression testing), 11 correct Bootstrap ARIA patterns Sonar misflags</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Medium (Minor)</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="18" t="n">
         <v>368</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="18" t="n">
         <v>353</v>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="18" t="inlineStr">
         <is>
           <t>Essentially cleared — mostly trailing whitespace and 101 real Subresource-Integrity hashes added to CDN scripts</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Info (Low)</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr">
         <is>
           <t>None were ever open</t>
         </is>
@@ -1094,282 +1664,282 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>Removed dead/commented-out code (backend + frontend)</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>Zero behavior change; code was already inert</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>CORS wildcard origin</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>Restricted to APP_URL; confirmed only affects an unused default /api/* stub route</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>50 duplicate HTML id attributes across 8 Blade views</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D13" s="18" t="inlineStr">
         <is>
           <t>Renamed to unique ids; cross-checked against all JS to confirm nothing was silently broken</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>101 CDN scripts/styles missing Subresource Integrity (SRI)</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="18" t="n">
         <v>101</v>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>Fetched exact bytes from each version-pinned CDN URL and computed real sha384 hashes</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>3 CDN resources without SRI (SweetAlert2, TinyMCE, html2canvas)</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>URLs are NOT version-pinned (e.g. .../tinymce/6/...) — a hardcoded hash would work today and silently break the app the next time that CDN updates its 'latest' build</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Invalid scope="row" attribute on &lt;td&gt; elements</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>HTML spec only allows scope on &lt;th&gt;; purely invalid markup, zero effect either way</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>Trailing whitespace / missing final newlines</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>~260</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>Purely mechanical, zero risk</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Form &lt;select&gt; elements not linked to a visible label</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>Linked via aria-labelledby to the real adjacent label cell instead of a copy-pasted Bootstrap-docs placeholder</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Logout link using href="javascript:void()" + onclick</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B19" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>Converted to a real &lt;button&gt;; tested logout end-to-end afterward</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>CSS font-family missing generic fallback</t>
         </is>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="15" t="n">
         <v>361</v>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>Won't fix</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>All are icon-font glyph declarations (Line Awesome, Material Design Icons, remixicon) — a generic fallback is meaningless for icon glyphs</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Duplicate CSS selectors/properties in vendor plugin files</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="15" t="inlineStr">
         <is>
           <t>Won't fix</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>Spread across 15+ third-party UI plugins (calendar, charts, editor...); merging risks silently changing cascade order with no way to visually regression-test each widget</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Prefer native &lt;progress&gt;/&lt;button&gt; over ARIA role</t>
         </is>
       </c>
-      <c r="B22" s="10" t="n">
+      <c r="B22" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>Won't fix</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>These are Bootstrap's own official patterns; swapping elements would require rebuilding CSS styling from scratch for a cosmetic lint preference</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>Commented code inside vendor icon-font file</t>
         </is>
       </c>
-      <c r="B23" s="10" t="n">
+      <c r="B23" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C23" s="15" t="inlineStr">
         <is>
           <t>Won't fix</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>26,000-line auto-generated stylesheet, explicitly marked 'Not included in production' by the upstream library</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Empty CSS comments (rtlcss directives)</t>
         </is>
       </c>
-      <c r="B24" s="10" t="n">
+      <c r="B24" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>Won't fix</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>These are /*rtl:begin:ignore*/ build directives controlling right-to-left layout for this app's Arabic locale — removing them breaks RTL support</t>
         </is>
@@ -1384,7 +1954,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1448,180 +2018,180 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="n">
+      <c r="A4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Invoice creation fails (HTTP 500) on every single submission</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>invoice.ewaybilldate column referenced by the app code has never existed in the database</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Added the missing nullable DATE column via ALTER TABLE (DB predates Laravel migrations, so a migration file wasn't the right mechanism here)</t>
         </is>
       </c>
-      <c r="F4" s="12" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Created a real invoice through the actual form end-to-end — succeeded</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Recording a payment against an invoice fails (HTTP 500)</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>InvoiceController.php calls Paidamount::create() with no `use App\Models\Paidamount;` import — PHP resolved the bare class name to a non-existent class in the Controllers namespace</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Added the missing import statement</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Recorded a real payment via the actual endpoint — invoice paid/remaining amount updated correctly</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="n">
+      <c r="A6" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Requested</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>Vendor page fails (HTTP 500)</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Query joined on invoice.customer_id, a column that doesn't exist — the real relationship is backwards (customer.invoice_id → invoice.id). Also never selected customer.name at all</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>Fixed join direction and added the missing name column to the select list</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Page renders 200 and correctly displays real customer names and invoice numbers</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="n">
+      <c r="A7" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Requested</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Invoice Details page fails (HTTP 500)</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Query selected product.product, a column that doesn't exist — the real column is product.name</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Aliased product.name AS product — required zero Blade template changes</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>Page renders 200 and correctly displays the real product name on a real invoice</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Every product created through the UI silently saves with a blank name</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Product::$fillable listed 'product'; the actual form field (and the actual database column) is 'name'. Laravel's mass-assignment protection silently drops any field not in $fillable — no error, just missing data</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Corrected the fillable array to list 'name'</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>Reproduced the bug live (submitted a real form, confirmed NULL saved), then confirmed the same submission saves correctly after the fix</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="n">
+      <c r="A9" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>CNC thickness values entered on the Technical Parameters page never save</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>Same bug class as #5 — Cnsthinks::$fillable had a typo ('cnsthinks') that matched neither the real form field name nor the real column name (both are 'cuttingthinks')</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>Corrected the fillable array</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="18" t="inlineStr">
         <is>
           <t>Reproduced and confirmed fixed the same way as #5</t>
         </is>
@@ -1636,7 +2206,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1688,482 +2258,482 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Dashboard / home</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr"/>
+      <c r="D4" s="18" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>/product</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Product list</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr"/>
+      <c r="D5" s="18" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>/apps-invoices-list</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Invoice list</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr"/>
+      <c r="D6" s="18" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>/apps-invoices-create</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Invoice creation form</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr"/>
+      <c r="D7" s="18" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>/invoiceddetails/{id}</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Invoice details view</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Fixed this session (bug #4)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>/paymenthistry</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Payment history list</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr"/>
+      <c r="D9" s="18" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>/vender</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>Vendor/customer list</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>Fixed this session (bug #3)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>/inventrylist</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>Inventory list</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr"/>
+      <c r="D11" s="18" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>/standerconfig/{id}</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>Product standard config page</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr"/>
+      <c r="D12" s="18" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>/standerconfiglist/{id}</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>Standard config list page</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr"/>
+      <c r="D13" s="18" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>/TechnicalParameters/{id}</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>Technical parameters page</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr"/>
+      <c r="D14" s="18" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>/fiberqutation/{id}</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>Fiber laser quotation form</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr"/>
+      <c r="D15" s="18" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>/admin/listqutation</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>Quotation list</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr"/>
+      <c r="D16" s="18" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>/printquation/{id}</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>Quotation PDF view</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr"/>
+      <c r="D17" s="18" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>/admin/invoice/getproductvalue</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>AJAX: get product value</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr"/>
+      <c r="D18" s="18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>/admin/invoice/getproduct1 (with param)</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>AJAX: get product value (variant)</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>Initial 500 was a missing test parameter, not a bug</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>/register, /password/reset</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>Auth utility pages</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr"/>
+      <c r="D20" s="18" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>/softerwere/{id}</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Add-software modal target view</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Pre-existing: returns view without required $id — see Known Issues sheet</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>/softerwere/show</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Software listing show-page</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Pre-existing: same missing-$id class of bug</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>/cutting/show</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Laser cutting show-page</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Pre-existing: controller method cuttingshow() was never implemented</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>/focusing/show</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Focusing show-page</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Pre-existing: controller method focusingshow() was never implemented</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>/power/show</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Power show-page</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>Pre-existing: controller method powershow() was never implemented</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>/cuttingway/{id}</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Cutting way detail view</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>Pre-existing: missing-$id class of bug</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>/co2quation</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>CO2 laser quotation form</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Pre-existing: shadowed by the app's catch-all route + controller requires an id the route never supplies</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="n"/>
+      <c r="A28" s="22" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="A29" s="22" t="inlineStr">
         <is>
           <t>Total routes tested</t>
         </is>
@@ -2173,7 +2743,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="22" t="inlineStr">
         <is>
           <t>Passing</t>
         </is>
@@ -2201,7 +2771,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2259,135 +2829,135 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>~10 'Add Software / Laser Cutting / Focusing / Power / Motor / Gear / Rack' modal forms error after submit</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>High — real data-entry forms inside the product config pages appear broken to users</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Each *store() method in StanderconfigController / StanderconfiglistController / TechinalController returns view('standerconfig') without passing the $id the view requires — 'Undefined variable $id'</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Touches ~10 call sites across 3 controllers; the correct fix (likely passing $request-&gt;input('product_id')) should be confirmed per call site rather than batch-patched</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>Fix each call site, passing the correct id; add a regression test per modal</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>3 dead routes: cutting/show, focusing/show, power/show</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>Routes point to StanderconfigController@cuttingshow / focusingshow / powershow — none of these three methods were ever implemented (only softerwereshow exists)</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Requires deciding what these pages should actually show — not a one-line fix</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Either implement the 3 missing methods or remove the dead routes, depending on product intent</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>co2quation route is unreachable</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Shadowed by the app's catch-all {any} route (registered earlier in routes/web.php), and the controller method requires an $id the route never supplies</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Found in an earlier session; fixing requires route re-ordering plus a route-signature decision</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Move the route above the catch-all and add the missing {id} parameter</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Laser Cutting Machine 'description' field never saves</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Low-Medium</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Three-way mismatch: the form sends 'details', the model's $fillable says 'description', the real database column is 'decription' (typo baked into the original table)</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Fixing the model alone won't fix this — the form field itself also needs to change; needs a decision on the intended canonical field name</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Decide the correct field name, then update form + model together</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Userdata model is fully dead code</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>None currently</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>Points at a table ('user', singular) that doesn't match its own $fillable columns, and nothing in the app references this model anywhere</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>Zero real-world impact since it's unused — not worth touching</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>Safe to delete if confirmed unused, or leave as-is</t>
         </is>

</xml_diff>